<commit_message>
String Tracker: columns match the string counts array
StudentName, 5+ Strings, 4-Strings, 3-Strings, 2-Strings, 1-Strings,
TotalUniqueCounters. Only the hidden String Tracker sheet changed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NCKyY7HhH1YBjfwnNdmgFF
</commit_message>
<xml_diff>
--- a/MasterData.xlsx
+++ b/MasterData.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="416">
   <si>
     <t>SyllabusID</t>
   </si>
@@ -1267,6 +1267,12 @@
   </si>
   <si>
     <t>IFT 41</t>
+  </si>
+  <si>
+    <t>5+ Strings</t>
+  </si>
+  <si>
+    <t>4-Strings</t>
   </si>
 </sst>
 </file>
@@ -2176,13 +2182,12 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.57421875" customWidth="1"/>
-    <col min="2" max="2" width="21.8515625" customWidth="1"/>
-    <col min="3" max="5" width="10.00390625" customWidth="1"/>
-    <col min="6" max="6" width="11.140625" customWidth="1"/>
+    <col min="2" max="6" width="10.00390625" customWidth="1"/>
+    <col min="7" max="7" width="21.8515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2190,19 +2195,22 @@
         <v>317</v>
       </c>
       <c r="B1" s="0" t="s">
+        <v>414</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>415</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>321</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>320</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>319</v>
+      </c>
+      <c r="G1" s="0" t="s">
         <v>318</v>
-      </c>
-      <c r="C1" s="0" t="s">
-        <v>319</v>
-      </c>
-      <c r="D1" s="0" t="s">
-        <v>320</v>
-      </c>
-      <c r="E1" s="0" t="s">
-        <v>321</v>
-      </c>
-      <c r="F1" s="0" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="2">
@@ -2224,6 +2232,9 @@
       <c r="F2" s="0">
         <v>0</v>
       </c>
+      <c r="G2" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
@@ -2244,6 +2255,9 @@
       <c r="F3" s="0">
         <v>0</v>
       </c>
+      <c r="G3" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
@@ -2264,6 +2278,9 @@
       <c r="F4" s="0">
         <v>0</v>
       </c>
+      <c r="G4" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
@@ -2284,6 +2301,9 @@
       <c r="F5" s="0">
         <v>0</v>
       </c>
+      <c r="G5" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
@@ -2304,6 +2324,9 @@
       <c r="F6" s="0">
         <v>0</v>
       </c>
+      <c r="G6" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
@@ -2324,6 +2347,9 @@
       <c r="F7" s="0">
         <v>0</v>
       </c>
+      <c r="G7" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
@@ -2344,6 +2370,9 @@
       <c r="F8" s="0">
         <v>0</v>
       </c>
+      <c r="G8" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
@@ -2364,6 +2393,9 @@
       <c r="F9" s="0">
         <v>0</v>
       </c>
+      <c r="G9" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
@@ -2384,6 +2416,9 @@
       <c r="F10" s="0">
         <v>0</v>
       </c>
+      <c r="G10" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
@@ -2404,6 +2439,9 @@
       <c r="F11" s="0">
         <v>0</v>
       </c>
+      <c r="G11" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
@@ -2424,6 +2462,9 @@
       <c r="F12" s="0">
         <v>0</v>
       </c>
+      <c r="G12" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
@@ -2444,6 +2485,9 @@
       <c r="F13" s="0">
         <v>0</v>
       </c>
+      <c r="G13" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
@@ -2462,6 +2506,9 @@
         <v>0</v>
       </c>
       <c r="F14" s="0">
+        <v>0</v>
+      </c>
+      <c r="G14" s="0">
         <v>0</v>
       </c>
     </row>

</xml_diff>